<commit_message>
fix google sheets source and frontend cache bust
</commit_message>
<xml_diff>
--- a/Equipos.xlsx
+++ b/Equipos.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RentAdvisor\Desktop\ChatBot Nyce\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ainsp-my.sharepoint.com/personal/brandon_trujillo_nycecolombia_co/Documents/ChatBot Nyce/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E4BA07C-4E2F-4766-81AB-FA31A7E91FD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2E7368C-691E-4B53-A9EC-FDBC1BBD3CD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4291,7 +4291,7 @@
       <c r="B4" s="56"/>
       <c r="C4" s="57">
         <f ca="1">TODAY()</f>
-        <v>46213</v>
+        <v>46218</v>
       </c>
       <c r="D4"/>
       <c r="E4" s="7"/>
@@ -14004,7 +14004,7 @@
       </c>
       <c r="S165" s="18" t="str">
         <f t="shared" ca="1" si="16"/>
-        <v>PROGRAMADO</v>
+        <v>VENCIDO</v>
       </c>
       <c r="T165" s="18" t="s">
         <v>34</v>
@@ -16857,7 +16857,7 @@
       <c r="B4" s="56"/>
       <c r="C4" s="57">
         <f ca="1">TODAY()</f>
-        <v>46213</v>
+        <v>46218</v>
       </c>
       <c r="D4"/>
       <c r="E4" s="7"/>
@@ -23574,7 +23574,7 @@
       <c r="B4" s="10"/>
       <c r="C4" s="11">
         <f ca="1">TODAY()</f>
-        <v>46213</v>
+        <v>46218</v>
       </c>
       <c r="D4"/>
       <c r="E4" s="7"/>
@@ -24007,7 +24007,7 @@
       <c r="B4" s="10"/>
       <c r="C4" s="11">
         <f ca="1">TODAY()</f>
-        <v>46213</v>
+        <v>46218</v>
       </c>
       <c r="D4"/>
       <c r="E4" s="7"/>
@@ -25023,56 +25023,6 @@
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
-<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10001</Type>
-    <SequenceNumber>1000</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10002</Type>
-    <SequenceNumber>1001</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10004</Type>
-    <SequenceNumber>1002</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10006</Type>
-    <SequenceNumber>1003</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-</spe:Receivers>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
@@ -25080,7 +25030,7 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <_dlc_DocId xmlns="b7b054a4-dd31-4e65-954f-c1858aefac91">VKQAY4435H2F-1852729036-123579</_dlc_DocId>
@@ -25096,7 +25046,7 @@
 </p:properties>
 </file>
 
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100FE666ABAACE12B4AB09E3E55549CF2E3" ma:contentTypeVersion="24" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="78d69b171ce51aea8268576e8ea78fd2">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b7b054a4-dd31-4e65-954f-c1858aefac91" xmlns:ns3="27dbd028-21f4-488b-a712-80beb6535a3a" xmlns:ns4="28fb201e-a7c2-4508-ac89-a084faf410d9" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b0dce42dc31ef7e3272b9c43bd330696" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="b7b054a4-dd31-4e65-954f-c1858aefac91"/>
@@ -25367,15 +25317,57 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{849E83F9-2C31-47D3-9A02-0DF4E45A9744}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10001</Type>
+    <SequenceNumber>1000</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10002</Type>
+    <SequenceNumber>1001</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10004</Type>
+    <SequenceNumber>1002</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10006</Type>
+    <SequenceNumber>1003</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+</spe:Receivers>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B869C843-68DD-4426-8D63-8D25788EB6A8}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
@@ -25383,7 +25375,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CAE72517-6D82-4507-8D0A-C885A2DF18D2}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -25394,7 +25386,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{21B2BBA1-4B08-4DB6-97E0-6021DE514217}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -25412,4 +25404,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{849E83F9-2C31-47D3-9A02-0DF4E45A9744}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>